<commit_message>
Update Figure 4 sweep labels and captions in source data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1g9vByMLTE8eGJ9K81zt6
</commit_message>
<xml_diff>
--- a/deliver/SourceData.xlsx
+++ b/deliver/SourceData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-1185" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figure 3a" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,12 +21,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 2" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 3" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 1" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 3" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 4b" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 5" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 7a,b" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 7c,d" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 3" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 5" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 6b" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 7" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 9a,b" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 9c,d" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="24" state="visible" r:id="rId24"/>
@@ -75,7 +75,12 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -109,9 +114,14 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2964,7 +2974,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Model parameters used in the Zn biodegradation simulation. The simulations used diffusivities 15-26% above the tabulated values (mm^2 h^-1: Zn2+ 3.38, Cl- 9.7, OH- 25.45, O2 10.8) and a film tortuosity of 120.</t>
+          <t>Model parameters used in the Zn biodegradation simulation.</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3028,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[46]</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3050,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[46]</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3082,7 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[47]</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3104,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[47]</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3126,7 @@
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[47]</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3148,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>[34]</t>
+          <t>[48]</t>
         </is>
       </c>
     </row>
@@ -3165,12 +3175,12 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>3.998 g cm^-3</t>
+          <t>5.606 g cm^-3</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[47]</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3200,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>[35]</t>
+          <t>[49]</t>
         </is>
       </c>
     </row>
@@ -3206,11 +3216,11 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>[36]</t>
+          <t>[50]</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3242,7 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>[33]</t>
+          <t>[46]</t>
         </is>
       </c>
     </row>
@@ -3247,10 +3257,26 @@
       <c r="D18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n"/>
-      <c r="B19" s="1" t="n"/>
-      <c r="C19" s="1" t="n"/>
-      <c r="D19" s="1" t="n"/>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Zn2+ sat. concentration</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>[Zn]_sat</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>10 mg L^-1</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>[51]</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3291,12 +3317,12 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>142.3 mmol L^-1 (5.04e-6 g mm^-3)</t>
+          <t>142.3 mmol L^-1</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>[38]</t>
+          <t>[52]</t>
         </is>
       </c>
     </row>
@@ -3313,12 +3339,12 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>3.5 mg L^-1 (3.5e-9 g mm^-3)</t>
+          <t>3.5 mg L^-1</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>[21]</t>
+          <t>[29]</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3364,7 @@
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>[39]</t>
+          <t>[53]</t>
         </is>
       </c>
     </row>
@@ -3411,13 +3437,11 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>[1, 1e5]</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>[v4 optimum]</t>
-        </is>
+          <t>[1, 100]</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>35.91</v>
       </c>
     </row>
     <row r="6">
@@ -3428,18 +3452,16 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>mm^6 g^-2 h^-1</t>
+          <t>L^2 mol^-2 h^-1</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>[8.0e6, 8.0e11]</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>[v4 optimum]</t>
-        </is>
+          <t>[5, 100]</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>27.17</v>
       </c>
     </row>
     <row r="7">
@@ -3455,13 +3477,11 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>[0.5, 50]</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>[v4 optimum]</t>
-        </is>
+          <t>[0.05, 5.0]</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.51</v>
       </c>
     </row>
     <row r="8">
@@ -3636,7 +3656,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 1</t>
+          <t>Supplementary Figure 3</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3667,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -3827,7 +3846,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 3</t>
+          <t>Supplementary Figure 5</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3857,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -5121,7 +5139,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 4b</t>
+          <t>Supplementary Figure 6b</t>
         </is>
       </c>
     </row>
@@ -5139,7 +5157,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -5930,7 +5947,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 5</t>
+          <t>Supplementary Figure 7</t>
         </is>
       </c>
     </row>
@@ -5941,7 +5958,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -10061,7 +10077,6 @@
       </c>
       <c r="H174" s="1" t="n"/>
     </row>
-    <row r="175"/>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
@@ -10957,14 +10972,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
@@ -10986,13 +11000,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Kinetic parameters: k_f = 35.91 h^-1, k_d = 27.17 L^2 mol^-2 h^-1, k_ORR = 0.51 mm h^-1 (calibrated optimum, Table 2).</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -11029,6 +11036,12 @@
           <t>Stage</t>
         </is>
       </c>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="M4" s="10" t="n"/>
+      <c r="N4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -11037,14 +11050,18 @@
       <c r="B5" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>35.90583</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>27.16962</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>0.50747</v>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>3.0×10⁵</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>1.0×10⁸</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>80</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>0.042402</v>
@@ -11054,6 +11071,12 @@
           <t>dip</t>
         </is>
       </c>
+      <c r="I5" s="11" t="n"/>
+      <c r="J5" s="11" t="n"/>
+      <c r="K5" s="11" t="n"/>
+      <c r="L5" s="11" t="n"/>
+      <c r="M5" s="11" t="n"/>
+      <c r="N5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -11062,14 +11085,18 @@
       <c r="B6" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>11.869081</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>36.881722</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>0.2513</v>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>9.9×10⁴</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>1.4×10⁸</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>40</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0.04609</v>
@@ -11079,6 +11106,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I6" s="11" t="n"/>
+      <c r="J6" s="11" t="n"/>
+      <c r="K6" s="11" t="n"/>
+      <c r="L6" s="11" t="n"/>
+      <c r="M6" s="11" t="n"/>
+      <c r="N6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -11087,14 +11120,18 @@
       <c r="B7" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>30.214196</v>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>61.694967</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>0.394269</v>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>2.5×10⁵</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>2.3×10⁸</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>62</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0.046374</v>
@@ -11104,6 +11141,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -11112,14 +11155,18 @@
       <c r="B8" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>48.4118</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>29.5251</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>0.5962</v>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>4.0×10⁵</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>1.1×10⁸</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>94</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>0.046388</v>
@@ -11129,6 +11176,12 @@
           <t>dip</t>
         </is>
       </c>
+      <c r="I8" s="11" t="n"/>
+      <c r="J8" s="11" t="n"/>
+      <c r="K8" s="11" t="n"/>
+      <c r="L8" s="11" t="n"/>
+      <c r="M8" s="11" t="n"/>
+      <c r="N8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -11137,14 +11190,18 @@
       <c r="B9" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="C9" s="1" t="n">
-        <v>57.872716</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>21.341167</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>0.656898</v>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>4.8×10⁵</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>7.9×10⁷</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>100</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>0.046866</v>
@@ -11154,6 +11211,12 @@
           <t>dip</t>
         </is>
       </c>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
+      <c r="M9" s="11" t="n"/>
+      <c r="N9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -11162,14 +11225,18 @@
       <c r="B10" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="C10" s="1" t="n">
-        <v>36.548579</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>14.595382</v>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>0.427188</v>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>3.1×10⁵</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>5.4×10⁷</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>67</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0.04719</v>
@@ -11179,6 +11246,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I10" s="11" t="n"/>
+      <c r="J10" s="11" t="n"/>
+      <c r="K10" s="11" t="n"/>
+      <c r="L10" s="11" t="n"/>
+      <c r="M10" s="11" t="n"/>
+      <c r="N10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -11187,14 +11260,18 @@
       <c r="B11" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="C11" s="1" t="n">
-        <v>51.43335</v>
-      </c>
-      <c r="D11" s="1" t="n">
-        <v>37.009824</v>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>0.704924</v>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>4.3×10⁵</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>1.4×10⁸</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>110</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>0.048462</v>
@@ -11204,6 +11281,12 @@
           <t>dip</t>
         </is>
       </c>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="N11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -11212,14 +11295,18 @@
       <c r="B12" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="1" t="n">
-        <v>4.364803</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>5.5078</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>0.15547</v>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>3.6×10⁴</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>2.0×10⁷</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>25</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>0.052771</v>
@@ -11229,6 +11316,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I12" s="11" t="n"/>
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="11" t="n"/>
+      <c r="M12" s="11" t="n"/>
+      <c r="N12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -11237,14 +11330,18 @@
       <c r="B13" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="C13" s="1" t="n">
-        <v>57.141068</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>42.489062</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>0.437817</v>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>4.8×10⁵</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>1.6×10⁸</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>69</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>0.055936</v>
@@ -11254,6 +11351,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
+      <c r="N13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -11262,14 +11365,18 @@
       <c r="B14" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="C14" s="1" t="n">
-        <v>57.480181</v>
-      </c>
-      <c r="D14" s="1" t="n">
-        <v>18.053204</v>
-      </c>
-      <c r="E14" s="1" t="n">
-        <v>0.434372</v>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>4.8×10⁵</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>6.6×10⁷</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>68</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>0.056486</v>
@@ -11279,6 +11386,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="11" t="n"/>
+      <c r="L14" s="11" t="n"/>
+      <c r="M14" s="11" t="n"/>
+      <c r="N14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -11287,14 +11400,18 @@
       <c r="B15" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="C15" s="1" t="n">
-        <v>66.021243</v>
-      </c>
-      <c r="D15" s="1" t="n">
-        <v>11.767734</v>
-      </c>
-      <c r="E15" s="1" t="n">
-        <v>0.452399</v>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>5.5×10⁵</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>4.3×10⁷</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>71</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0.05756</v>
@@ -11304,6 +11421,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
+      <c r="M15" s="11" t="n"/>
+      <c r="N15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -11312,14 +11435,18 @@
       <c r="B16" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="C16" s="1" t="n">
-        <v>58.226265</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>0.430407</v>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>4.9×10⁵</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>3.7×10⁸</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>68</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>0.057868</v>
@@ -11329,6 +11456,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I16" s="11" t="n"/>
+      <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="n"/>
+      <c r="N16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -11337,14 +11470,18 @@
       <c r="B17" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="C17" s="1" t="n">
-        <v>60.640234</v>
-      </c>
-      <c r="D17" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E17" s="1" t="n">
-        <v>0.433336</v>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>5.1×10⁵</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>1.8×10⁷</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>68</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>0.058507</v>
@@ -11354,6 +11491,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="11" t="n"/>
+      <c r="N17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -11362,14 +11505,18 @@
       <c r="B18" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="C18" s="1" t="n">
-        <v>66.116321</v>
-      </c>
-      <c r="D18" s="1" t="n">
-        <v>27.695915</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>0.445382</v>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>5.5×10⁵</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>1.0×10⁸</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>70</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>0.058528</v>
@@ -11379,6 +11526,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -11387,14 +11540,18 @@
       <c r="B19" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="C19" s="1" t="n">
-        <v>60.154809</v>
-      </c>
-      <c r="D19" s="1" t="n">
-        <v>7.670637</v>
-      </c>
-      <c r="E19" s="1" t="n">
-        <v>0.431341</v>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>5.0×10⁵</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>2.8×10⁷</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>68</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0.059043</v>
@@ -11404,6 +11561,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I19" s="11" t="n"/>
+      <c r="J19" s="11" t="n"/>
+      <c r="K19" s="11" t="n"/>
+      <c r="L19" s="11" t="n"/>
+      <c r="M19" s="11" t="n"/>
+      <c r="N19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -11412,14 +11575,18 @@
       <c r="B20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="C20" s="1" t="n">
-        <v>55.129743</v>
-      </c>
-      <c r="D20" s="1" t="n">
-        <v>65.183634</v>
-      </c>
-      <c r="E20" s="1" t="n">
-        <v>0.418043</v>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>4.6×10⁵</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>2.4×10⁸</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>66</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0.059716</v>
@@ -11429,6 +11596,12 @@
           <t>phase2</t>
         </is>
       </c>
+      <c r="I20" s="11" t="n"/>
+      <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="11" t="n"/>
+      <c r="M20" s="11" t="n"/>
+      <c r="N20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -11437,14 +11610,18 @@
       <c r="B21" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="C21" s="1" t="n">
-        <v>6.248831</v>
-      </c>
-      <c r="D21" s="1" t="n">
-        <v>12.592237</v>
-      </c>
-      <c r="E21" s="1" t="n">
-        <v>0.165976</v>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>5.2×10⁴</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>4.6×10⁷</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>26</v>
       </c>
       <c r="F21" s="1" t="n">
         <v>0.060445</v>
@@ -11454,6 +11631,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -11462,14 +11645,18 @@
       <c r="B22" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="C22" s="1" t="n">
-        <v>14.726772</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>47.756723</v>
-      </c>
-      <c r="E22" s="1" t="n">
-        <v>0.526387</v>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>1.2×10⁵</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>1.8×10⁸</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>83</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>0.070782</v>
@@ -11479,6 +11666,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
+      <c r="N22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -11487,14 +11680,18 @@
       <c r="B23" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="C23" s="1" t="n">
-        <v>25.55777</v>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>28.358274</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>0.705943</v>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>2.1×10⁵</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>1.0×10⁸</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>110</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>0.07711800000000001</v>
@@ -11504,6 +11701,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I23" s="11" t="n"/>
+      <c r="J23" s="11" t="n"/>
+      <c r="K23" s="11" t="n"/>
+      <c r="L23" s="11" t="n"/>
+      <c r="M23" s="11" t="n"/>
+      <c r="N23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -11512,14 +11715,18 @@
       <c r="B24" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="C24" s="1" t="n">
-        <v>62.647707</v>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>13.264881</v>
-      </c>
-      <c r="E24" s="1" t="n">
-        <v>0.301923</v>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>5.2×10⁵</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>4.9×10⁷</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>48</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>0.088184</v>
@@ -11529,6 +11736,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -11537,14 +11750,18 @@
       <c r="B25" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C25" s="1" t="n">
-        <v>1.694926</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>48.516168</v>
-      </c>
-      <c r="E25" s="1" t="n">
-        <v>0.079988</v>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>1.4×10⁴</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>1.8×10⁸</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>13</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>0.100601</v>
@@ -11554,6 +11771,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I25" s="11" t="n"/>
+      <c r="J25" s="11" t="n"/>
+      <c r="K25" s="11" t="n"/>
+      <c r="L25" s="11" t="n"/>
+      <c r="M25" s="11" t="n"/>
+      <c r="N25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -11562,14 +11785,18 @@
       <c r="B26" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="C26" s="1" t="n">
-        <v>50.313013</v>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>39.610909</v>
-      </c>
-      <c r="E26" s="1" t="n">
-        <v>1.082887</v>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>4.2×10⁵</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>1.5×10⁸</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>170</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>0.100613</v>
@@ -11579,6 +11806,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I26" s="11" t="n"/>
+      <c r="J26" s="11" t="n"/>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="11" t="n"/>
+      <c r="M26" s="11" t="n"/>
+      <c r="N26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -11587,14 +11820,18 @@
       <c r="B27" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="C27" s="1" t="n">
-        <v>21.406276</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>20.22353</v>
-      </c>
-      <c r="E27" s="1" t="n">
-        <v>0.820634</v>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>1.8×10⁵</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>7.4×10⁷</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>130</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>0.112077</v>
@@ -11604,6 +11841,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I27" s="11" t="n"/>
+      <c r="J27" s="11" t="n"/>
+      <c r="K27" s="11" t="n"/>
+      <c r="L27" s="11" t="n"/>
+      <c r="M27" s="11" t="n"/>
+      <c r="N27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -11612,14 +11855,18 @@
       <c r="B28" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="C28" s="1" t="n">
-        <v>75.720311</v>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>22.601489</v>
-      </c>
-      <c r="E28" s="1" t="n">
-        <v>0.222116</v>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>6.3×10⁵</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>8.3×10⁷</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>35</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>0.112735</v>
@@ -11629,6 +11876,12 @@
           <t>phase3</t>
         </is>
       </c>
+      <c r="I28" s="11" t="n"/>
+      <c r="J28" s="11" t="n"/>
+      <c r="K28" s="11" t="n"/>
+      <c r="L28" s="11" t="n"/>
+      <c r="M28" s="11" t="n"/>
+      <c r="N28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -11637,14 +11890,18 @@
       <c r="B29" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="1" t="n">
-        <v>19.536874</v>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>20.009222</v>
-      </c>
-      <c r="E29" s="1" t="n">
-        <v>0.887589</v>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>1.6×10⁵</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>7.4×10⁷</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>140</v>
       </c>
       <c r="F29" s="1" t="n">
         <v>0.126677</v>
@@ -11654,6 +11911,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I29" s="11" t="n"/>
+      <c r="J29" s="11" t="n"/>
+      <c r="K29" s="11" t="n"/>
+      <c r="L29" s="11" t="n"/>
+      <c r="M29" s="11" t="n"/>
+      <c r="N29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -11662,14 +11925,18 @@
       <c r="B30" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C30" s="1" t="n">
-        <v>32.64415</v>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>24.529234</v>
-      </c>
-      <c r="E30" s="1" t="n">
-        <v>0.060249</v>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>2.7×10⁵</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>9.0×10⁷</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="n">
+        <v>9.5</v>
       </c>
       <c r="F30" s="1" t="n">
         <v>0.154122</v>
@@ -11679,6 +11946,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I30" s="11" t="n"/>
+      <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
+      <c r="M30" s="11" t="n"/>
+      <c r="N30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -11687,14 +11960,18 @@
       <c r="B31" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="C31" s="1" t="n">
-        <v>2.937196</v>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>65.546769</v>
-      </c>
-      <c r="E31" s="1" t="n">
-        <v>0.462952</v>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>2.5×10⁴</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>2.4×10⁸</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="n">
+        <v>73</v>
       </c>
       <c r="F31" s="1" t="n">
         <v>0.160994</v>
@@ -11704,6 +11981,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="n"/>
+      <c r="N31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -11712,14 +11995,18 @@
       <c r="B32" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C32" s="1" t="n">
-        <v>67.991682</v>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>8.613716999999999</v>
-      </c>
-      <c r="E32" s="1" t="n">
-        <v>2.508756</v>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>5.7×10⁵</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>3.2×10⁷</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>400</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>0.206768</v>
@@ -11729,6 +12016,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I32" s="11" t="n"/>
+      <c r="J32" s="11" t="n"/>
+      <c r="K32" s="11" t="n"/>
+      <c r="L32" s="11" t="n"/>
+      <c r="M32" s="11" t="n"/>
+      <c r="N32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -11737,14 +12030,18 @@
       <c r="B33" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C33" s="1" t="n">
-        <v>24.90597</v>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>78.122794</v>
-      </c>
-      <c r="E33" s="1" t="n">
-        <v>2.136741</v>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>2.1×10⁵</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>2.9×10⁸</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>340</v>
       </c>
       <c r="F33" s="1" t="n">
         <v>0.260444</v>
@@ -11754,6 +12051,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I33" s="11" t="n"/>
+      <c r="J33" s="11" t="n"/>
+      <c r="K33" s="11" t="n"/>
+      <c r="L33" s="11" t="n"/>
+      <c r="M33" s="11" t="n"/>
+      <c r="N33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -11762,14 +12065,18 @@
       <c r="B34" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C34" s="1" t="n">
-        <v>9.864005000000001</v>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>15.319409</v>
-      </c>
-      <c r="E34" s="1" t="n">
-        <v>1.322114</v>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>8.2×10⁴</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>5.6×10⁷</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>210</v>
       </c>
       <c r="F34" s="1" t="n">
         <v>0.276129</v>
@@ -11779,6 +12086,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n"/>
+      <c r="L34" s="11" t="n"/>
+      <c r="M34" s="11" t="n"/>
+      <c r="N34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -11787,14 +12100,18 @@
       <c r="B35" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C35" s="1" t="n">
-        <v>83.562388</v>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>34.156142</v>
-      </c>
-      <c r="E35" s="1" t="n">
-        <v>4.493303</v>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>7.0×10⁵</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>1.3×10⁸</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>710</v>
       </c>
       <c r="F35" s="1" t="n">
         <v>0.307616</v>
@@ -11804,6 +12121,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I35" s="11" t="n"/>
+      <c r="J35" s="11" t="n"/>
+      <c r="K35" s="11" t="n"/>
+      <c r="L35" s="11" t="n"/>
+      <c r="M35" s="11" t="n"/>
+      <c r="N35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -11812,14 +12135,18 @@
       <c r="B36" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="C36" s="1" t="n">
-        <v>1.212982</v>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>7.744136</v>
-      </c>
-      <c r="E36" s="1" t="n">
-        <v>0.730585</v>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>1.0×10⁴</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>2.9×10⁷</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="n">
+        <v>120</v>
       </c>
       <c r="F36" s="1" t="n">
         <v>0.320861</v>
@@ -11829,6 +12156,12 @@
           <t>global</t>
         </is>
       </c>
+      <c r="I36" s="11" t="n"/>
+      <c r="J36" s="11" t="n"/>
+      <c r="K36" s="11" t="n"/>
+      <c r="L36" s="11" t="n"/>
+      <c r="M36" s="11" t="n"/>
+      <c r="N36" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11847,7 +12180,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 7a,b</t>
+          <t>Supplementary Figure 9a,b</t>
         </is>
       </c>
     </row>
@@ -11858,7 +12191,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -15790,7 +16122,6 @@
         <v>3.411422</v>
       </c>
     </row>
-    <row r="175"/>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
@@ -15885,7 +16216,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 7c,d</t>
+          <t>Supplementary Figure 9c,d</t>
         </is>
       </c>
     </row>
@@ -15896,7 +16227,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -16042,7 +16372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16051,85 +16381,94 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Table S1</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Limiting regimes of the interfacial oxygen flux.</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Comparison of the candidate velocity-selection formulations. Rule A (hard minimum) best matched literature mass-loss measurements and was adopted in the final model.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Regime</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Interfacial flux J_O2</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>RMSE (%)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Reaction-controlled</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Da &lt;&lt; 1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>k_ORR C_b</t>
-        </is>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Hard minimum</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.0568</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Transition</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Da ~ 1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>C_b/(1/k_ORR + delta/D_O2,eff)</t>
-        </is>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Mixed control</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.077</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Diffusion-controlled</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Da &gt;&gt; 1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>D_O2,eff C_b/delta</t>
-        </is>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Hybrid cathodic</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.0766</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Coupled ORR (no O2 cap)</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.2983</v>
       </c>
     </row>
   </sheetData>
@@ -16162,7 +16501,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Mesh convergence study showing the effect of mesh resolution on predicted 7-day mass loss. Relative errors are calculated with respect to the reference mesh.</t>
+          <t>Mesh convergence study showing the effect of mesh resolution on predicted 7-day mass loss. Relative errors are calculated with respect to the reference mesh (21.25 million elements).</t>
         </is>
       </c>
     </row>
@@ -16189,114 +16528,114 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>L1 (Very Low)</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="9" t="n">
         <v>182768</v>
       </c>
-      <c r="C5" t="n">
-        <v>0.3009</v>
-      </c>
-      <c r="D5" t="n">
-        <v>87.2</v>
+      <c r="C5" s="7" t="n">
+        <v>1.439</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>1465.8</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>L2 (Low)</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="9" t="n">
         <v>802365</v>
       </c>
-      <c r="C6" t="n">
-        <v>0.2029</v>
-      </c>
-      <c r="D6" t="n">
-        <v>26.2</v>
+      <c r="C6" s="6" t="n">
+        <v>0.4977</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>441.6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>L3 (Medium)</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="9" t="n">
         <v>3454723</v>
       </c>
-      <c r="C7" t="n">
-        <v>0.1682</v>
-      </c>
-      <c r="D7" t="n">
-        <v>4.6</v>
+      <c r="C7" s="6" t="n">
+        <v>0.1633</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>77.7</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>L4 (High)</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="9" t="n">
         <v>4990080</v>
       </c>
-      <c r="C8" t="n">
-        <v>0.1637</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1.8</v>
+      <c r="C8" s="6" t="n">
+        <v>0.1208</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>31.4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>L5 (Very High)</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="9" t="n">
         <v>11958220</v>
       </c>
-      <c r="C9" t="n">
-        <v>0.1616</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.5</v>
+      <c r="C9" s="6" t="n">
+        <v>0.1002</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>L6 (Ultra High)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="9" t="n">
         <v>18864900</v>
       </c>
-      <c r="C10" t="n">
-        <v>0.1611</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.19</v>
+      <c r="C10" s="6" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.87</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="9" t="n">
         <v>21245850</v>
       </c>
-      <c r="C11" t="n">
-        <v>0.1608</v>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C11" s="6" t="n">
+        <v>0.0919</v>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -16333,7 +16672,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Comparison between an adaptive mesh and a uniform mesh (approximately 800,000 elements).</t>
+          <t>Comparison between adaptive and uniform meshes at approximately 800,000 elements.</t>
         </is>
       </c>
     </row>
@@ -16365,63 +16704,63 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Uniform Mesh</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>799000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.286</v>
-      </c>
-      <c r="D5" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="B5" s="9" t="n">
+        <v>799520</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>2.8561</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>3007.8</v>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Adaptive Mesh</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="9" t="n">
         <v>802365</v>
       </c>
-      <c r="C6" t="n">
-        <v>0.2029</v>
-      </c>
-      <c r="D6" t="n">
-        <v>26.2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.663</v>
+      <c r="C6" s="6" t="n">
+        <v>0.4977</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>441.6</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.8532</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Reference Mesh</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="9" t="n">
         <v>21245850</v>
       </c>
-      <c r="C7" t="n">
-        <v>0.1608</v>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C7" s="6" t="n">
+        <v>0.0919</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -16440,9 +16779,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16707,7 +17044,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>37,399</t>
+          <t>802,365</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
@@ -16729,7 +17066,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>[to update]</t>
+          <t>121,120</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
@@ -16751,7 +17088,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>0.5 mm</t>
+          <t>0.1 mm</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -16827,7 +17164,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>4 h</t>
+          <t>0.25 h</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
@@ -16902,7 +17239,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>50</v>
@@ -16919,7 +17256,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>[to update]</t>
+          <t>2,592</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
@@ -17029,7 +17366,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>~20 min</t>
+          <t>2 h</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
@@ -17137,7 +17474,7 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>Dirichlet (C_O2 = 3.5 mg L^-1)</t>
+          <t>Dirichlet</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
@@ -17203,7 +17540,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Parameters included in the Morris sensitivity analysis (the ranges might differ from calibration space as this was done prior to calibration of the model).</t>
+          <t>Parameters included in the Morris sensitivity analysis.</t>
         </is>
       </c>
     </row>
@@ -17805,7 +18142,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Mass-loss response (%) to one-at-a-time parameter sweeps of k_f (panel a), k_d (panel b), and k_ORR (panel c). Baseline: k_f = 35, k_d = 27, k_ORR = 0.5 (middle curves).</t>
+          <t>Mass-loss response (%) to one-at-a-time parameter sweeps of k_f (panel a), k_d (panel b), and k_ORR (panel c). Baseline: k_f = 3.0×10⁵ h⁻¹, k_d = 1.0×10⁸ mm⁶ g⁻² h⁻¹, k_ORR = 80 mm h⁻¹ (middle curves); low/high = 0.13×/3.3× (k_f), 0.2×/4× (k_d), 0.2×/5× (k_ORR).</t>
         </is>
       </c>
     </row>
@@ -17824,17 +18161,17 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>kf 5</t>
+          <t>kf 4.0×10⁴</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>kf 35</t>
+          <t>kf 3.0×10⁵</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>kf 150</t>
+          <t>kf 1.0×10⁶</t>
         </is>
       </c>
     </row>
@@ -18448,17 +18785,17 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>kd 5</t>
+          <t>kd 2.0×10⁷</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>kd 27</t>
+          <t>kd 1.0×10⁸</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>kd 120</t>
+          <t>kd 4.0×10⁸</t>
         </is>
       </c>
     </row>
@@ -19072,17 +19409,17 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.1</t>
+          <t>kORR 16</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.5</t>
+          <t>kORR 80</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>kORR 2.5</t>
+          <t>kORR 400</t>
         </is>
       </c>
     </row>
@@ -20046,8 +20383,7 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20598,7 +20934,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Corrosion-product saturation, F/Fmax (%), in one-at-a-time parameter sweeps of k_f (panel d), k_d (panel e), and k_ORR (panel f). Baseline: k_f = 35, k_d = 27, k_ORR = 0.5 (middle curves).</t>
+          <t>Corrosion-product saturation, F/Fmax (%), in one-at-a-time parameter sweeps of k_f (panel d), k_d (panel e), and k_ORR (panel f). Baseline: k_f = 3.0×10⁵ h⁻¹, k_d = 1.0×10⁸ mm⁶ g⁻² h⁻¹, k_ORR = 80 mm h⁻¹ (middle curves); low/high = 0.13×/3.3× (k_f), 0.2×/4× (k_d), 0.2×/5× (k_ORR).</t>
         </is>
       </c>
     </row>
@@ -20617,17 +20953,17 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>kf 5</t>
+          <t>kf 4.0×10⁴</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>kf 35</t>
+          <t>kf 3.0×10⁵</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>kf 150</t>
+          <t>kf 1.0×10⁶</t>
         </is>
       </c>
     </row>
@@ -21241,17 +21577,17 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>kd 5</t>
+          <t>kd 2.0×10⁷</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>kd 27</t>
+          <t>kd 1.0×10⁸</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>kd 120</t>
+          <t>kd 4.0×10⁸</t>
         </is>
       </c>
     </row>
@@ -21865,17 +22201,17 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.1</t>
+          <t>kORR 16</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.5</t>
+          <t>kORR 80</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>kORR 2.5</t>
+          <t>kORR 400</t>
         </is>
       </c>
     </row>
@@ -22505,7 +22841,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Interfacial dissolved oxygen concentration response (mg/L) to one-at-a-time parameter sweeps of k_f (panel g), k_d (panel h), and k_ORR (panel i). Baseline: k_f = 35, k_d = 27, k_ORR = 0.5 (middle curves).</t>
+          <t>Interfacial dissolved oxygen concentration response (mg/L) to one-at-a-time parameter sweeps of k_f (panel g), k_d (panel h), and k_ORR (panel i). Baseline: k_f = 3.0×10⁵ h⁻¹, k_d = 1.0×10⁸ mm⁶ g⁻² h⁻¹, k_ORR = 80 mm h⁻¹ (middle curves); low/high = 0.13×/3.3× (k_f), 0.2×/4× (k_d), 0.2×/5× (k_ORR).</t>
         </is>
       </c>
     </row>
@@ -22524,17 +22860,17 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>kf 5</t>
+          <t>kf 4.0×10⁴</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>kf 35</t>
+          <t>kf 3.0×10⁵</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>kf 150</t>
+          <t>kf 1.0×10⁶</t>
         </is>
       </c>
     </row>
@@ -23148,17 +23484,17 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>kd 5</t>
+          <t>kd 2.0×10⁷</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>kd 27</t>
+          <t>kd 1.0×10⁸</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>kd 120</t>
+          <t>kd 4.0×10⁸</t>
         </is>
       </c>
     </row>
@@ -23772,17 +24108,17 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.1</t>
+          <t>kORR 16</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>kORR 0.5</t>
+          <t>kORR 80</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>kORR 2.5</t>
+          <t>kORR 400</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SI figure renumbering (tracked) and source-data sheet names
</commit_message>
<xml_diff>
--- a/deliver/SourceData.xlsx
+++ b/deliver/SourceData.xlsx
@@ -21,12 +21,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 2" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 3" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 3" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 5" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 6b" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 7" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 9a,b" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 9c,d" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 1" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 3" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 4b" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 6" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 8a,b" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 8c,d" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 10a" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplementary Figure 10b" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="24" state="visible" r:id="rId24"/>
@@ -3658,7 +3658,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 3</t>
+          <t>Supplementary Figure 1</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 5</t>
+          <t>Supplementary Figure 3</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 6b</t>
+          <t>Supplementary Figure 4b</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5949,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 7</t>
+          <t>Supplementary Figure 6</t>
         </is>
       </c>
     </row>
@@ -12182,7 +12182,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 9a,b</t>
+          <t>Supplementary Figure 8a,b</t>
         </is>
       </c>
     </row>
@@ -16218,7 +16218,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Supplementary Figure 9c,d</t>
+          <t>Supplementary Figure 8c,d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final validation: cross-reference fixes, caption numbering, Excel sync, validation report
</commit_message>
<xml_diff>
--- a/deliver/SourceData.xlsx
+++ b/deliver/SourceData.xlsx
@@ -2957,7 +2957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3008,12 +3008,12 @@
           <t>Material properties</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n"/>
-      <c r="C5" s="1" t="n"/>
-      <c r="D5" s="1" t="n"/>
+      <c r="B5" s="1" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
+      <c r="D5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Zn density</t>
         </is>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>[46]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Zn molar mass</t>
         </is>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>[46]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
@@ -3062,12 +3062,12 @@
           <t>Diffusion coefficients (37 °C)</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n"/>
-      <c r="C8" s="1" t="n"/>
-      <c r="D8" s="1" t="n"/>
+      <c r="B8" s="1" t="inlineStr"/>
+      <c r="C8" s="1" t="inlineStr"/>
+      <c r="D8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Zn2+ diffusivity</t>
         </is>
@@ -3084,12 +3084,12 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>[47]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Cl- diffusivity</t>
         </is>
@@ -3106,12 +3106,12 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>[47]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>OH- diffusivity</t>
         </is>
@@ -3128,12 +3128,12 @@
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>[47]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>O2 diffusivity</t>
         </is>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>[48]</t>
+          <t>[33]</t>
         </is>
       </c>
     </row>
@@ -3160,12 +3160,12 @@
           <t>Film properties</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="1" t="n"/>
-      <c r="D13" s="1" t="n"/>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Film density</t>
         </is>
@@ -3182,12 +3182,12 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>[47]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Film porosity</t>
         </is>
@@ -3197,17 +3197,19 @@
           <t>ε</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
-        <v>0.25</v>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>[49]</t>
+          <t>[34]</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Film tortuosity</t>
         </is>
@@ -3217,17 +3219,19 @@
           <t>τ</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
-        <v>2</v>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>[50]</t>
+          <t>[35]</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Film molar mass</t>
         </is>
@@ -3244,129 +3248,101 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>[46]</t>
+          <t>[32]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Interface conditions</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
+          <t>Initial conditions</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Zn2+ sat. concentration</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Zn2+ concentration</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>[Zn]_sat</t>
+          <t>C_Zn^0</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>10 mg L^-1</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>[51]</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Initial conditions</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="n"/>
-      <c r="C20" s="1" t="n"/>
-      <c r="D20" s="1" t="n"/>
+          <t>Cl- concentration</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>C_Cl^0</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>1.42 × 10^-7 mol mm^-3</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>[36]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Zn2+ concentration</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>O2 concentration</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>C_Zn^0</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="1" t="n"/>
+          <t>C_O2^0</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>1.09 × 10^-10 mol mm^-3</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>[21]</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Cl- concentration</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>pH</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>C_Cl^0</t>
+          <t>–</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>142.3 mmol L^-1</t>
+          <t>7.40</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>[52]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>O2 concentration</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>C_O2^0</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>3.5 mg L^-1</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>[29]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>pH</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>[53]</t>
+          <t>[37]</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3439,11 +3415,13 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>[1, 100]</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>35.91</v>
+          <t>[1×10⁴, 8×10⁵]</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>3×10⁵</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3454,16 +3432,18 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>L^2 mol^-2 h^-1</t>
+          <t>mm^6 g^-2 h^-1</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>[5, 100]</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>27.17</v>
+          <t>[2×10⁷, 4×10⁸]</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1×10⁸</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -3474,36 +3454,18 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>mm h^-1 (effective)</t>
+          <t>mm h^-1</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>[0.05, 5.0]</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>M_O2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>g mol^-1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>32</v>
+          <t>[8, 800]</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -21731,7 +21693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21749,85 +21711,76 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Comparison of the candidate velocity-selection formulations. Rule A (hard minimum) best matched literature mass-loss measurements and was adopted in the final model.</t>
+          <t>Limiting regimes of the interfacial oxygen flux.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Rule</t>
+          <t>Regime</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Condition</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>RMSE (%)</t>
+          <t>Interfacial flux J_O₂</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Reaction-controlled</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Hard minimum</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>0.0568</v>
+          <t>Da ≪ 1</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>k_ORR C_b</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Transition</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Mixed control</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>0.077</v>
+          <t>Da ≈ 1</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>C_b /(1/k_ORR + δ/D_O₂,eff)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Diffusion-controlled</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Hybrid cathodic</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>0.0766</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Coupled ORR (no O2 cap)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>0.2983</v>
+          <t>Da ≫ 1</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>D_O₂,eff C_b /δ</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -21860,7 +21813,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Mesh convergence study showing the effect of mesh resolution on predicted 7-day mass loss. Relative errors are calculated with respect to the reference mesh (21.25 million elements).</t>
+          <t>Mesh convergence study showing the effect of mesh resolution on predicted 7-day mass loss. Relative errors are calculated with respect to the reference mesh (Mass Loss values may differ from those of the calibrated model, as these validation cases were evaluated prior to model calibration).</t>
         </is>
       </c>
     </row>
@@ -21896,10 +21849,10 @@
         <v>182768</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1.439</v>
+        <v>0.3009</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1465.8</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="6">
@@ -21911,11 +21864,11 @@
       <c r="B6" s="9" t="n">
         <v>802365</v>
       </c>
-      <c r="C6" s="6" t="n">
-        <v>0.4977</v>
+      <c r="C6" s="7" t="n">
+        <v>0.2029</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>441.6</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="7">
@@ -21927,11 +21880,11 @@
       <c r="B7" s="9" t="n">
         <v>3454723</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>0.1633</v>
+      <c r="C7" s="7" t="n">
+        <v>0.1682</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>77.7</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="8">
@@ -21943,11 +21896,11 @@
       <c r="B8" s="9" t="n">
         <v>4990080</v>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>0.1208</v>
+      <c r="C8" s="7" t="n">
+        <v>0.1637</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>31.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9">
@@ -21959,11 +21912,11 @@
       <c r="B9" s="9" t="n">
         <v>11958220</v>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>0.1002</v>
+      <c r="C9" s="7" t="n">
+        <v>0.1616</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>9</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
@@ -21975,11 +21928,11 @@
       <c r="B10" s="9" t="n">
         <v>18864900</v>
       </c>
-      <c r="C10" s="6" t="n">
-        <v>0.0927</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0.87</v>
+      <c r="C10" s="7" t="n">
+        <v>0.1611</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>0.19</v>
       </c>
     </row>
     <row r="11">
@@ -21991,10 +21944,10 @@
       <c r="B11" s="9" t="n">
         <v>21245850</v>
       </c>
-      <c r="C11" s="6" t="n">
-        <v>0.0919</v>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="C11" s="7" t="n">
+        <v>0.1608</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -22031,7 +21984,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Comparison between adaptive and uniform meshes at approximately 800,000 elements.</t>
+          <t>Comparison between an adaptive mesh and a uniform mesh (approximately 800,000 elements).</t>
         </is>
       </c>
     </row>
@@ -22069,13 +22022,13 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>799520</v>
+        <v>799000</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2.8561</v>
+        <v>0.286</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>3007.8</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
@@ -22093,13 +22046,13 @@
         <v>802365</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>0.4977</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>441.6</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>0.8532</v>
+        <v>0.2029</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0.663</v>
       </c>
     </row>
     <row r="7">
@@ -22112,14 +22065,14 @@
         <v>21245850</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.0919</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
+        <v>0.1608</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -22452,7 +22405,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>0.04 mm</t>
+          <t>0.005 mm</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -22598,7 +22551,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>50</v>
@@ -22899,7 +22852,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Parameters included in the Morris sensitivity analysis.</t>
+          <t>Parameters included in the Morris sensitivity analysis (the ranges might differ from calibration space as this was done prior to calibration of the model).</t>
         </is>
       </c>
     </row>
@@ -22938,7 +22891,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>50–200</t>
+          <t>1×10⁴ – 8×10⁵</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -22960,7 +22913,7 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>1–50</t>
+          <t>2×10⁷ – 4×10⁸</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
@@ -22982,7 +22935,7 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>0.1–5.0</t>
+          <t>8 – 800</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -23026,7 +22979,7 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1×10^-9 to 1×10^-7</t>
+          <t>1×10^-9 – 1×10^-8</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -25157,7 +25110,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Literature mass-loss data used for Bayesian calibration (Liu et al. 2018).</t>
+          <t>Literature mass-loss data used for calibration (Liu et al. 2018).</t>
         </is>
       </c>
     </row>
@@ -25755,7 +25708,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Comparison of simulated and measured mass loss in HBSS (validation) with the experimental scatter. Experimental values are mean ± SD (n = 3).</t>
+          <t>Comparison of simulated and measured mass loss in HBSS (validation) with the experimental scatter. Experimental values are mean ± SD (n = 3); |Error|/SD is the absolute error divided by the SD at the same immersion time. The validation RMSE of 0.0159% (R² = 0.9734) corresponds to 8.6% of the mean measured mass loss (0.185%) and 5.1% of the 28-day value.</t>
         </is>
       </c>
     </row>
@@ -25963,7 +25916,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Geometric and computational parameters of the controlled test structures used in Figure 8.</t>
+          <t>Geometric and computational parameters of the controlled test structures used in main-text Figure 8.</t>
         </is>
       </c>
     </row>

</xml_diff>